<commit_message>
[Product] - Add turnover class validation and update checkbox handling in mass update product functionality
</commit_message>
<xml_diff>
--- a/public/upload/template/mass_update_product.xlsx
+++ b/public/upload/template/mass_update_product.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9FFD3756-22CC-4ACA-BA4F-814BF07C378E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D3D33A4-0CF8-4061-BDAA-B4D49303E84F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{DB2DEC0F-61AA-4766-BB0D-92993A6FF919}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="34">
   <si>
     <t>article_id</t>
   </si>
@@ -134,6 +134,9 @@
   </si>
   <si>
     <t>p_turnoverclass</t>
+  </si>
+  <si>
+    <t>NON MOVING, SLOW MOVING, FAST MOVING</t>
   </si>
 </sst>
 </file>
@@ -520,7 +523,7 @@
   <cols>
     <col min="1" max="1" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.77734375" customWidth="1"/>
-    <col min="3" max="3" width="20.21875" customWidth="1"/>
+    <col min="3" max="3" width="39.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -729,7 +732,7 @@
         <v>7</v>
       </c>
       <c r="C19" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Products] - add SKU level update for sell price
</commit_message>
<xml_diff>
--- a/public/upload/template/mass_update_product.xlsx
+++ b/public/upload/template/mass_update_product.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D3D33A4-0CF8-4061-BDAA-B4D49303E84F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22A628B8-D92D-45FB-A732-B88CFA5C3111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{DB2DEC0F-61AA-4766-BB0D-92993A6FF919}"/>
   </bookViews>
   <sheets>
-    <sheet name="Ini Yang di import" sheetId="1" r:id="rId1"/>
-    <sheet name="kolom yang bisa diganti" sheetId="2" r:id="rId2"/>
+    <sheet name="Article Level" sheetId="1" r:id="rId1"/>
+    <sheet name="SKU Level" sheetId="3" r:id="rId2"/>
+    <sheet name="kolom yang bisa diganti" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="36">
   <si>
     <t>article_id</t>
   </si>
@@ -137,6 +138,12 @@
   </si>
   <si>
     <t>NON MOVING, SLOW MOVING, FAST MOVING</t>
+  </si>
+  <si>
+    <t>ps_sell_price</t>
+  </si>
+  <si>
+    <t>ps_barcode</t>
   </si>
 </sst>
 </file>
@@ -517,6 +524,28 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E9C748E-38DF-4768-B6DC-D1BD889CD343}">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.77734375" customWidth="1"/>
+    <col min="2" max="2" width="24.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB8AE581-1C2B-49F7-AE37-C0E7CD7C6D0E}">
   <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
[Products] - change mass update file
</commit_message>
<xml_diff>
--- a/public/upload/template/mass_update_product.xlsx
+++ b/public/upload/template/mass_update_product.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2717b52d0fafc363/Documents/From D/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22A628B8-D92D-45FB-A732-B88CFA5C3111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{22A628B8-D92D-45FB-A732-B88CFA5C3111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C566E84-C1DA-4013-8784-6A728FE8975B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{DB2DEC0F-61AA-4766-BB0D-92993A6FF919}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{DB2DEC0F-61AA-4766-BB0D-92993A6FF919}"/>
   </bookViews>
   <sheets>
     <sheet name="Article Level" sheetId="1" r:id="rId1"/>
@@ -116,9 +116,6 @@
     <t>mp_best_seller</t>
   </si>
   <si>
-    <t>complemenet</t>
-  </si>
-  <si>
     <t>consigment</t>
   </si>
   <si>
@@ -144,6 +141,9 @@
   </si>
   <si>
     <t>ps_barcode</t>
+  </si>
+  <si>
+    <t>complement</t>
   </si>
 </sst>
 </file>
@@ -534,10 +534,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -689,7 +689,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B13" t="s">
         <v>24</v>
@@ -700,7 +700,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B14" t="s">
         <v>24</v>
@@ -711,7 +711,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
         <v>24</v>
@@ -722,7 +722,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B16" t="s">
         <v>24</v>
@@ -733,7 +733,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17" t="s">
         <v>24</v>
@@ -744,7 +744,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B18" t="s">
         <v>24</v>
@@ -755,13 +755,13 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B19" t="s">
         <v>7</v>
       </c>
       <c r="C19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Product] - add mark down flag
</commit_message>
<xml_diff>
--- a/public/upload/template/mass_update_product.xlsx
+++ b/public/upload/template/mass_update_product.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2717b52d0fafc363/Documents/From D/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{22A628B8-D92D-45FB-A732-B88CFA5C3111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C566E84-C1DA-4013-8784-6A728FE8975B}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{22A628B8-D92D-45FB-A732-B88CFA5C3111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B193D46-4206-496D-9FDA-40FFE86E63EA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{DB2DEC0F-61AA-4766-BB0D-92993A6FF919}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="37">
   <si>
     <t>article_id</t>
   </si>
@@ -144,6 +144,9 @@
   </si>
   <si>
     <t>complement</t>
+  </si>
+  <si>
+    <t>mark_down</t>
   </si>
 </sst>
 </file>
@@ -547,7 +550,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB8AE581-1C2B-49F7-AE37-C0E7CD7C6D0E}">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.5546875" bestFit="1" customWidth="1"/>
@@ -764,6 +767,17 @@
         <v>32</v>
       </c>
     </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>36</v>
+      </c>
+      <c r="B20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
[Product] - fix mass update consignment
</commit_message>
<xml_diff>
--- a/public/upload/template/mass_update_product.xlsx
+++ b/public/upload/template/mass_update_product.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2717b52d0fafc363/Documents/From D/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PecelAfrika\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{22A628B8-D92D-45FB-A732-B88CFA5C3111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B193D46-4206-496D-9FDA-40FFE86E63EA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{645FAFE0-5557-475E-955C-467BC57F6C53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{DB2DEC0F-61AA-4766-BB0D-92993A6FF919}"/>
   </bookViews>
@@ -116,9 +116,6 @@
     <t>mp_best_seller</t>
   </si>
   <si>
-    <t>consigment</t>
-  </si>
-  <si>
     <t>mp_stock_masking</t>
   </si>
   <si>
@@ -147,6 +144,9 @@
   </si>
   <si>
     <t>mark_down</t>
+  </si>
+  <si>
+    <t>consignment</t>
   </si>
 </sst>
 </file>
@@ -537,10 +537,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -692,7 +692,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
         <v>24</v>
@@ -703,7 +703,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="B14" t="s">
         <v>24</v>
@@ -714,7 +714,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B15" t="s">
         <v>24</v>
@@ -725,7 +725,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
         <v>24</v>
@@ -736,7 +736,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B17" t="s">
         <v>24</v>
@@ -747,7 +747,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B18" t="s">
         <v>24</v>
@@ -758,18 +758,18 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B19" t="s">
         <v>7</v>
       </c>
       <c r="C19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B20" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
[Product] - add ability to mass update price tag on sku level
</commit_message>
<xml_diff>
--- a/public/upload/template/mass_update_product.xlsx
+++ b/public/upload/template/mass_update_product.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PecelAfrika\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IT1\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{645FAFE0-5557-475E-955C-467BC57F6C53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37490079-AE45-4227-A6AE-C673897DC14B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{DB2DEC0F-61AA-4766-BB0D-92993A6FF919}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{DB2DEC0F-61AA-4766-BB0D-92993A6FF919}"/>
   </bookViews>
   <sheets>
     <sheet name="Article Level" sheetId="1" r:id="rId1"/>
@@ -25,10 +25,7 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -134,9 +131,6 @@
     <t>NON MOVING, SLOW MOVING, FAST MOVING</t>
   </si>
   <si>
-    <t>ps_sell_price</t>
-  </si>
-  <si>
     <t>ps_barcode</t>
   </si>
   <si>
@@ -147,6 +141,9 @@
   </si>
   <si>
     <t>consignment</t>
+  </si>
+  <si>
+    <t>ps_sell_price/ps_price_tag</t>
   </si>
 </sst>
 </file>
@@ -537,10 +534,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -692,7 +689,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B13" t="s">
         <v>24</v>
@@ -703,7 +700,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" t="s">
         <v>24</v>
@@ -769,7 +766,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B20" t="s">
         <v>24</v>

</xml_diff>